<commit_message>
Update DATA MASTER KONTRAK NO '7207250142.xlsx
</commit_message>
<xml_diff>
--- a/DATA MASTER KONTRAK NO '7207250142.xlsx
+++ b/DATA MASTER KONTRAK NO '7207250142.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\98 PROFORMA INVOICE\Dashboard Proforma Invoice General Services\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD39E97F-D247-41C6-8792-EF2A8EB4B503}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{645FA6B3-A551-4F5F-A439-780272D881A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" tabRatio="719" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -912,7 +912,7 @@
     <t>Kategori</t>
   </si>
   <si>
-    <t>Spesifikasi / Deskripsi Pekerjaan </t>
+    <t>Spesifikasi / Deskripsi Pekerjaan</t>
   </si>
 </sst>
 </file>
@@ -1636,7 +1636,7 @@
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="No." dataDxfId="9" dataCellStyle="Normal 3 3"/>
     <tableColumn id="8" xr3:uid="{EE801E05-357E-44F3-A601-DC0237DBA5BC}" name="No Kontrak" dataDxfId="8" dataCellStyle="Normal 3 3"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Kategori" dataDxfId="7" dataCellStyle="Normal 3 3"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Spesifikasi / Deskripsi Pekerjaan " dataDxfId="6" dataCellStyle="Normal 14"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Spesifikasi / Deskripsi Pekerjaan" dataDxfId="6" dataCellStyle="Normal 14"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Qty" dataDxfId="5" dataCellStyle="Normal 3 3"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Unit" dataDxfId="4" dataCellStyle="Normal 3 3"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Satuan" dataDxfId="3" dataCellStyle="Normal 3 3"/>

</xml_diff>